<commit_message>
modify file 1 và đăng ký file 2
</commit_message>
<xml_diff>
--- a/A/Github_Excel001.xlsx
+++ b/A/Github_Excel001.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\LinhLT\Job\02.Server_GIT\8352\8352_repoGithub001\A\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3032509B-DF51-4626-8F67-07CCC280C5F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3587D007-030C-4B41-A90D-2D611DB2FD7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3020" yWindow="-90" windowWidth="14580" windowHeight="10170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -165,7 +165,7 @@
     <t>C25</t>
   </si>
   <si>
-    <t>C26</t>
+    <t>C26_11</t>
   </si>
 </sst>
 </file>
@@ -187,12 +187,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -207,8 +213,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -702,7 +709,7 @@
       <c r="B26" t="s">
         <v>16</v>
       </c>
-      <c r="C26" t="s">
+      <c r="C26" s="1" t="s">
         <v>46</v>
       </c>
     </row>

</xml_diff>

<commit_message>
update nội dung file
</commit_message>
<xml_diff>
--- a/A/Github_Excel001.xlsx
+++ b/A/Github_Excel001.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\LinhLT\Job\02.Server_GIT\8352\8352_repoGithub001\A\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3587D007-030C-4B41-A90D-2D611DB2FD7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FC70D8C-5AA1-4A16-9095-8C096F82320A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -165,7 +165,7 @@
     <t>C25</t>
   </si>
   <si>
-    <t>C26_11</t>
+    <t>C26_13</t>
   </si>
 </sst>
 </file>

</xml_diff>